<commit_message>
Add project files and tests
</commit_message>
<xml_diff>
--- a/frontend/static/templates/Washing_Setup_Template.xlsx
+++ b/frontend/static/templates/Washing_Setup_Template.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -468,6 +468,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>For updates, blank cells mean leave the saved value as it is.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Remarks: the current situation at the plant (e.g. water tanker every 3 days, south gate locked on Sundays).</t>
         </is>
       </c>
     </row>
@@ -527,7 +534,7 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Remarks</t>
         </is>
       </c>
     </row>

</xml_diff>